<commit_message>
Built out skeleton environment examples to include worksheet, netcdf, and profile event list.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/skeleton/skeleton_v4.xlsx
+++ b/src/rattlesnake/examples/environment/skeleton/skeleton_v4.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Rattlesnake\rattlesnake-vibration-controller-dev\src\rattlesnake\examples\environment\skeleton\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller\src\rattlesnake\examples\environment\skeleton\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{371C386E-21AA-422B-B92C-8B3BA968F759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E454D2AB-3D7D-4D61-899E-92E77F708DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Skeleton 0" sheetId="4" r:id="rId1"/>
+    <sheet name="Test Profile" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t>Control Type</t>
   </si>
@@ -35,6 +36,57 @@
   </si>
   <si>
     <t># None type object used to show how to store example data to worksheets</t>
+  </si>
+  <si>
+    <t>Time (s)</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Operation</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>0.0</t>
+  </si>
+  <si>
+    <t>Global</t>
+  </si>
+  <si>
+    <t>Start Streaming</t>
+  </si>
+  <si>
+    <t>Skeleton 0</t>
+  </si>
+  <si>
+    <t>Start Environment</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>Example Set Test Level</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Example Float Command</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>Stop Environment</t>
+  </si>
+  <si>
+    <t>Stop Hardware</t>
   </si>
 </sst>
 </file>
@@ -402,4 +454,100 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C1078B4-3314-4066-950A-D67E0695CCA0}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>